<commit_message>
Merge macropage-connect and mrfuels-transact into one unified admin app
Replaces the two separate NestJS apps with a single apps/admin that
connects to both product databases at once (default connection for
macropage-connect, named 'mrFuels' connection for mr-fuels) and shares
one admin login across both. Routes are namespaced under
/api/macropage-connect/* and /api/mr-fuels/*.

Also adds macropage-connect help docs/FAQ CRUD (writes into the real
live helpdocs/helpfaqs collections), a tutorial upload endpoint backed
by DigitalOcean Spaces, fixes the plans catalog to mirror the real
portal's PLAN_PRICING instead of the internal Razorpay config, and
fixes a password/secret leak in the customers list response.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/macropage-connect-api.xlsx
+++ b/docs/macropage-connect-api.xlsx
@@ -3,11 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="macropage-connect APIs" sheetId="1" r:id="rId1"/>
+    <sheet name="macropage-connect API" sheetId="1" r:id="rId1"/>
     <sheet name="Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'macropage-connect APIs'!A1:G35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'macropage-connect API'!A1:H46</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,15 +401,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:H46"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="60.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="7.83203125" customWidth="1"/>
+    <col min="3" max="3" width="42.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="55.83203125" customWidth="1"/>
+    <col min="8" max="8" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -432,10 +433,13 @@
         <v>Request Body / Query Params</v>
       </c>
       <c r="G1" t="str">
+        <v>Example Payload</v>
+      </c>
+      <c r="H1" t="str">
         <v>Description</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>Auth</v>
       </c>
@@ -454,8 +458,14 @@
       <c r="F2" t="str">
         <v>{ email, password }</v>
       </c>
-      <c r="G2" t="str">
-        <v>Admin login — returns JWT accessToken + user info</v>
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "email": "admin@macropage.com",
+  "password": "change-me-123"
+}</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Admin login — returns { accessToken, user }. Same login works for /mr-fuels/* too.</v>
       </c>
     </row>
     <row r="3">
@@ -466,7 +476,7 @@
         <v>GET</v>
       </c>
       <c r="C3" t="str">
-        <v>/customers</v>
+        <v>/macropage-connect/customers</v>
       </c>
       <c r="D3" t="str">
         <v>JWT required</v>
@@ -475,10 +485,13 @@
         <v>Any</v>
       </c>
       <c r="F3" t="str">
-        <v>Query: page, limit, search, billingPlan, tagId</v>
+        <v>Query: page, limit, search, billingPlan(TRIAL|STARTER|GROWTH|BUSINESS|ENTERPRISE), tagId</v>
       </c>
       <c r="G3" t="str">
-        <v>Paginated list of customers (real "users" collection, role=OWNER)</v>
+        <v>-</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Paginated list (real "users" collection, role=OWNER)</v>
       </c>
     </row>
     <row r="4">
@@ -489,7 +502,7 @@
         <v>GET</v>
       </c>
       <c r="C4" t="str">
-        <v>/customers/:id</v>
+        <v>/macropage-connect/customers/:id</v>
       </c>
       <c r="D4" t="str">
         <v>JWT required</v>
@@ -501,7 +514,10 @@
         <v>-</v>
       </c>
       <c r="G4" t="str">
-        <v>Get one customer (password/secrets stripped)</v>
+        <v>-</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Get one customer (secrets stripped)</v>
       </c>
     </row>
     <row r="5">
@@ -512,7 +528,7 @@
         <v>GET</v>
       </c>
       <c r="C5" t="str">
-        <v>/customers/:id/profile</v>
+        <v>/macropage-connect/customers/:id/profile</v>
       </c>
       <c r="D5" t="str">
         <v>JWT required</v>
@@ -524,7 +540,10 @@
         <v>-</v>
       </c>
       <c r="G5" t="str">
-        <v>Full profile: customer + currentPlan + planHistory + messageStats + tags</v>
+        <v>-</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Returns { customer, currentPlan, planHistory, messageStats, tags }</v>
       </c>
     </row>
     <row r="6">
@@ -535,7 +554,7 @@
         <v>GET</v>
       </c>
       <c r="C6" t="str">
-        <v>/plans</v>
+        <v>/macropage-connect/plans</v>
       </c>
       <c r="D6" t="str">
         <v>JWT required</v>
@@ -547,7 +566,10 @@
         <v>-</v>
       </c>
       <c r="G6" t="str">
-        <v>Plan catalog (Starter/Growth/Business, hardcoded pricing)</v>
+        <v>-</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Portal pricing catalog (Starter/Growth/Scale/Enterprise, monthly/quarterly/yearly)</v>
       </c>
     </row>
     <row r="7">
@@ -558,7 +580,7 @@
         <v>GET</v>
       </c>
       <c r="C7" t="str">
-        <v>/plans/customer/:tenantId</v>
+        <v>/macropage-connect/plans/customer/:tenantId</v>
       </c>
       <c r="D7" t="str">
         <v>JWT required</v>
@@ -570,7 +592,10 @@
         <v>-</v>
       </c>
       <c r="G7" t="str">
-        <v>Purchase/renewal history for a customer (real payments collection)</v>
+        <v>-</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Purchase/renewal history (real payments collection)</v>
       </c>
     </row>
     <row r="8">
@@ -581,7 +606,7 @@
         <v>GET</v>
       </c>
       <c r="C8" t="str">
-        <v>/plans/customer/:tenantId/current</v>
+        <v>/macropage-connect/plans/customer/:tenantId/current</v>
       </c>
       <c r="D8" t="str">
         <v>JWT required</v>
@@ -593,7 +618,10 @@
         <v>-</v>
       </c>
       <c r="G8" t="str">
-        <v>Current active subscription for a customer</v>
+        <v>-</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Current active subscription</v>
       </c>
     </row>
     <row r="9">
@@ -604,7 +632,7 @@
         <v>GET</v>
       </c>
       <c r="C9" t="str">
-        <v>/messages/logs</v>
+        <v>/macropage-connect/messages/logs</v>
       </c>
       <c r="D9" t="str">
         <v>JWT required</v>
@@ -613,10 +641,13 @@
         <v>Any</v>
       </c>
       <c r="F9" t="str">
-        <v>Query: page, limit, customerId, status, from, to</v>
+        <v>Query: page, limit, customerId, status(PENDING|SENT|DELIVERED|READ|FAILED), from, to</v>
       </c>
       <c r="G9" t="str">
-        <v>Message send logs (real messages collection, direction=OUTBOUND)</v>
+        <v>-</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Message send logs (real messages, direction=OUTBOUND)</v>
       </c>
     </row>
     <row r="10">
@@ -627,7 +658,7 @@
         <v>GET</v>
       </c>
       <c r="C10" t="str">
-        <v>/messages/stats</v>
+        <v>/macropage-connect/messages/stats</v>
       </c>
       <c r="D10" t="str">
         <v>JWT required</v>
@@ -639,7 +670,10 @@
         <v>Query: customerId, groupBy(day|month), from, to</v>
       </c>
       <c r="G10" t="str">
-        <v>Message stats aggregated by day/month, sent/failed/total</v>
+        <v>-</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Sent/failed/total counts grouped by day or month</v>
       </c>
     </row>
     <row r="11">
@@ -650,7 +684,7 @@
         <v>GET</v>
       </c>
       <c r="C11" t="str">
-        <v>/tags</v>
+        <v>/macropage-connect/tags</v>
       </c>
       <c r="D11" t="str">
         <v>JWT required</v>
@@ -662,10 +696,13 @@
         <v>-</v>
       </c>
       <c r="G11" t="str">
-        <v>List all tags</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>-</v>
+      </c>
+      <c r="H11" t="str">
+        <v>List tags</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
       <c r="A12" t="str">
         <v>Tags</v>
       </c>
@@ -673,7 +710,7 @@
         <v>POST</v>
       </c>
       <c r="C12" t="str">
-        <v>/tags</v>
+        <v>/macropage-connect/tags</v>
       </c>
       <c r="D12" t="str">
         <v>JWT required</v>
@@ -684,11 +721,18 @@
       <c r="F12" t="str">
         <v>{ name, color?, description? }</v>
       </c>
-      <c r="G12" t="str">
-        <v>Create a tag</v>
-      </c>
-    </row>
-    <row r="13">
+      <c r="G12" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "name": "VIP",
+  "color": "#f97316",
+  "description": "High-value customers"
+}</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Create tag</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
       <c r="A13" t="str">
         <v>Tags</v>
       </c>
@@ -696,7 +740,7 @@
         <v>PATCH</v>
       </c>
       <c r="C13" t="str">
-        <v>/tags/:id</v>
+        <v>/macropage-connect/tags/:id</v>
       </c>
       <c r="D13" t="str">
         <v>JWT required</v>
@@ -707,8 +751,13 @@
       <c r="F13" t="str">
         <v>{ name?, color?, description? }</v>
       </c>
-      <c r="G13" t="str">
-        <v>Update a tag</v>
+      <c r="G13" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "color": "#22c55e"
+}</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Update tag</v>
       </c>
     </row>
     <row r="14">
@@ -719,7 +768,7 @@
         <v>DELETE</v>
       </c>
       <c r="C14" t="str">
-        <v>/tags/:id</v>
+        <v>/macropage-connect/tags/:id</v>
       </c>
       <c r="D14" t="str">
         <v>JWT required</v>
@@ -731,10 +780,13 @@
         <v>-</v>
       </c>
       <c r="G14" t="str">
-        <v>Delete a tag</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>-</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Delete tag</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
       <c r="A15" t="str">
         <v>Tags</v>
       </c>
@@ -742,7 +794,7 @@
         <v>POST</v>
       </c>
       <c r="C15" t="str">
-        <v>/tags/assign</v>
+        <v>/macropage-connect/tags/assign</v>
       </c>
       <c r="D15" t="str">
         <v>JWT required</v>
@@ -753,7 +805,15 @@
       <c r="F15" t="str">
         <v>{ customerId, tagIds: string[] }</v>
       </c>
-      <c r="G15" t="str">
+      <c r="G15" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "customerId": "665f1a2b9c1d4e0012345678",
+  "tagIds": [
+    "665f1a2b9c1d4e0012345aaa"
+  ]
+}</v>
+      </c>
+      <c r="H15" t="str">
         <v>Replace a customer's tag set</v>
       </c>
     </row>
@@ -765,7 +825,7 @@
         <v>GET</v>
       </c>
       <c r="C16" t="str">
-        <v>/templates</v>
+        <v>/macropage-connect/templates</v>
       </c>
       <c r="D16" t="str">
         <v>JWT required</v>
@@ -777,7 +837,10 @@
         <v>-</v>
       </c>
       <c r="G16" t="str">
-        <v>List notification templates (admin-owned, distinct from real WhatsApp templates)</v>
+        <v>-</v>
+      </c>
+      <c r="H16" t="str">
+        <v>List notification templates</v>
       </c>
     </row>
     <row r="17">
@@ -788,7 +851,7 @@
         <v>GET</v>
       </c>
       <c r="C17" t="str">
-        <v>/templates/:id</v>
+        <v>/macropage-connect/templates/:id</v>
       </c>
       <c r="D17" t="str">
         <v>JWT required</v>
@@ -800,10 +863,13 @@
         <v>-</v>
       </c>
       <c r="G17" t="str">
-        <v>Get one template</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>-</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Get one</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
       <c r="A18" t="str">
         <v>Templates</v>
       </c>
@@ -811,7 +877,7 @@
         <v>POST</v>
       </c>
       <c r="C18" t="str">
-        <v>/templates</v>
+        <v>/macropage-connect/templates</v>
       </c>
       <c r="D18" t="str">
         <v>JWT required</v>
@@ -822,11 +888,22 @@
       <c r="F18" t="str">
         <v>{ name, channel(whatsapp|sms|push), content, variables?: string[], isActive? }</v>
       </c>
-      <c r="G18" t="str">
-        <v>Create template ({{variable}} placeholders supported)</v>
-      </c>
-    </row>
-    <row r="19">
+      <c r="G18" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "name": "Welcome",
+  "channel": "whatsapp",
+  "content": "Hi {{name}}, welcome to Macropage!",
+  "variables": [
+    "name"
+  ],
+  "isActive": true
+}</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Create ({{variable}} placeholders supported)</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
       <c r="A19" t="str">
         <v>Templates</v>
       </c>
@@ -834,7 +911,7 @@
         <v>PATCH</v>
       </c>
       <c r="C19" t="str">
-        <v>/templates/:id</v>
+        <v>/macropage-connect/templates/:id</v>
       </c>
       <c r="D19" t="str">
         <v>JWT required</v>
@@ -845,8 +922,13 @@
       <c r="F19" t="str">
         <v>Partial of create body</v>
       </c>
-      <c r="G19" t="str">
-        <v>Update template</v>
+      <c r="G19" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "isActive": false
+}</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Update</v>
       </c>
     </row>
     <row r="20">
@@ -857,7 +939,7 @@
         <v>DELETE</v>
       </c>
       <c r="C20" t="str">
-        <v>/templates/:id</v>
+        <v>/macropage-connect/templates/:id</v>
       </c>
       <c r="D20" t="str">
         <v>JWT required</v>
@@ -869,7 +951,10 @@
         <v>-</v>
       </c>
       <c r="G20" t="str">
-        <v>Delete template</v>
+        <v>-</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Delete</v>
       </c>
     </row>
     <row r="21">
@@ -880,7 +965,7 @@
         <v>GET</v>
       </c>
       <c r="C21" t="str">
-        <v>/notifications</v>
+        <v>/macropage-connect/notifications</v>
       </c>
       <c r="D21" t="str">
         <v>JWT required</v>
@@ -892,10 +977,13 @@
         <v>-</v>
       </c>
       <c r="G21" t="str">
-        <v>List past admin broadcasts (send history)</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>-</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Broadcast send history</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
       <c r="A22" t="str">
         <v>Notifications</v>
       </c>
@@ -903,7 +991,7 @@
         <v>POST</v>
       </c>
       <c r="C22" t="str">
-        <v>/notifications/broadcast</v>
+        <v>/macropage-connect/notifications/broadcast</v>
       </c>
       <c r="D22" t="str">
         <v>JWT required</v>
@@ -914,11 +1002,18 @@
       <c r="F22" t="str">
         <v>{ title, body, channel(in_app|whatsapp) }</v>
       </c>
-      <c r="G22" t="str">
-        <v>Send to ALL customers; in_app writes into real notifications collection, whatsapp sends via Twilio</v>
-      </c>
-    </row>
-    <row r="23">
+      <c r="G22" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "title": "New feature!",
+  "body": "Bulk campaigns are now live.",
+  "channel": "in_app"
+}</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Send to ALL customers</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
       <c r="A23" t="str">
         <v>Notifications</v>
       </c>
@@ -926,7 +1021,7 @@
         <v>POST</v>
       </c>
       <c r="C23" t="str">
-        <v>/notifications/send</v>
+        <v>/macropage-connect/notifications/send</v>
       </c>
       <c r="D23" t="str">
         <v>JWT required</v>
@@ -935,9 +1030,20 @@
         <v>Any</v>
       </c>
       <c r="F23" t="str">
-        <v>{ title, body, channel(in_app|whatsapp), targetType(tag|customer), targetIds: string[] }</v>
-      </c>
-      <c r="G23" t="str">
+        <v>{ title, body, channel, targetType(tag|customer), targetIds: string[] }</v>
+      </c>
+      <c r="G23" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "title": "Renewal reminder",
+  "body": "Your plan expires in 3 days",
+  "channel": "whatsapp",
+  "targetType": "customer",
+  "targetIds": [
+    "665f1a2b9c1d4e0012345678"
+  ]
+}</v>
+      </c>
+      <c r="H23" t="str">
         <v>Send to specific tag(s) or customer(s)</v>
       </c>
     </row>
@@ -949,7 +1055,7 @@
         <v>GET</v>
       </c>
       <c r="C24" t="str">
-        <v>/ads</v>
+        <v>/macropage-connect/ads</v>
       </c>
       <c r="D24" t="str">
         <v>JWT required</v>
@@ -961,7 +1067,10 @@
         <v>-</v>
       </c>
       <c r="G24" t="str">
-        <v>List all ads/popups (admin view)</v>
+        <v>-</v>
+      </c>
+      <c r="H24" t="str">
+        <v>List all ads (admin view)</v>
       </c>
     </row>
     <row r="25">
@@ -972,7 +1081,7 @@
         <v>GET</v>
       </c>
       <c r="C25" t="str">
-        <v>/ads/active</v>
+        <v>/macropage-connect/ads/active</v>
       </c>
       <c r="D25" t="str">
         <v>JWT required</v>
@@ -984,10 +1093,13 @@
         <v>Query: customerId? (optional)</v>
       </c>
       <c r="G25" t="str">
-        <v>Currently-active ads, optionally targeted to one customer</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>-</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Currently-active ads</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
       <c r="A26" t="str">
         <v>Ads</v>
       </c>
@@ -995,7 +1107,7 @@
         <v>POST</v>
       </c>
       <c r="C26" t="str">
-        <v>/ads</v>
+        <v>/macropage-connect/ads</v>
       </c>
       <c r="D26" t="str">
         <v>JWT required</v>
@@ -1004,13 +1116,23 @@
         <v>Any</v>
       </c>
       <c r="F26" t="str">
-        <v>{ title, mediaUrl, type(popup|banner|inline), targetType?(all|tag|customer), targetIds?: string[], isActive?, startDate?, endDate?, priority? }</v>
-      </c>
-      <c r="G26" t="str">
+        <v>{ title, mediaUrl, type(popup|banner|inline), targetType?(all|tag|customer), targetIds?, isActive?, startDate?, endDate?, priority? }</v>
+      </c>
+      <c r="G26" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "title": "Diwali Offer",
+  "mediaUrl": "https://cdn.example.com/diwali.png",
+  "type": "popup",
+  "targetType": "all",
+  "isActive": true,
+  "priority": 10
+}</v>
+      </c>
+      <c r="H26" t="str">
         <v>Create an ad/popup</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" xml:space="preserve">
       <c r="A27" t="str">
         <v>Ads</v>
       </c>
@@ -1018,7 +1140,7 @@
         <v>PATCH</v>
       </c>
       <c r="C27" t="str">
-        <v>/ads/:id</v>
+        <v>/macropage-connect/ads/:id</v>
       </c>
       <c r="D27" t="str">
         <v>JWT required</v>
@@ -1029,8 +1151,13 @@
       <c r="F27" t="str">
         <v>Partial of create body</v>
       </c>
-      <c r="G27" t="str">
-        <v>Update an ad/popup</v>
+      <c r="G27" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "isActive": false
+}</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Update</v>
       </c>
     </row>
     <row r="28">
@@ -1041,7 +1168,7 @@
         <v>DELETE</v>
       </c>
       <c r="C28" t="str">
-        <v>/ads/:id</v>
+        <v>/macropage-connect/ads/:id</v>
       </c>
       <c r="D28" t="str">
         <v>JWT required</v>
@@ -1053,7 +1180,10 @@
         <v>-</v>
       </c>
       <c r="G28" t="str">
-        <v>Delete an ad/popup</v>
+        <v>-</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Delete</v>
       </c>
     </row>
     <row r="29">
@@ -1064,7 +1194,7 @@
         <v>GET</v>
       </c>
       <c r="C29" t="str">
-        <v>/stats/dashboard</v>
+        <v>/macropage-connect/stats/dashboard</v>
       </c>
       <c r="D29" t="str">
         <v>JWT required</v>
@@ -1076,18 +1206,21 @@
         <v>-</v>
       </c>
       <c r="G29" t="str">
-        <v>totalCustomers, totalEnrolledCustomers, messagesSentToday, messagesFailedToday</v>
+        <v>-</v>
+      </c>
+      <c r="H29" t="str">
+        <v>{ totalCustomers, totalEnrolledCustomers, messagesSentToday, messagesFailedToday }</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Support Tickets</v>
+        <v>Help Docs</v>
       </c>
       <c r="B30" t="str">
         <v>GET</v>
       </c>
       <c r="C30" t="str">
-        <v>/support/tickets</v>
+        <v>/macropage-connect/help/docs</v>
       </c>
       <c r="D30" t="str">
         <v>JWT required</v>
@@ -1096,21 +1229,24 @@
         <v>Any</v>
       </c>
       <c r="F30" t="str">
-        <v>Query: page, limit, status, priority, customerId, assignedTo</v>
+        <v>Query: category?</v>
       </c>
       <c r="G30" t="str">
-        <v>Paginated list of support tickets</v>
+        <v>-</v>
+      </c>
+      <c r="H30" t="str">
+        <v>List help docs (real, live helpdocs collection)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Support Tickets</v>
+        <v>Help Docs</v>
       </c>
       <c r="B31" t="str">
         <v>GET</v>
       </c>
       <c r="C31" t="str">
-        <v>/support/tickets/:id</v>
+        <v>/macropage-connect/help/docs/:id</v>
       </c>
       <c r="D31" t="str">
         <v>JWT required</v>
@@ -1122,18 +1258,21 @@
         <v>-</v>
       </c>
       <c r="G31" t="str">
-        <v>Get one ticket</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>-</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Get one</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
       <c r="A32" t="str">
-        <v>Support Tickets</v>
+        <v>Help Docs</v>
       </c>
       <c r="B32" t="str">
         <v>POST</v>
       </c>
       <c r="C32" t="str">
-        <v>/support/tickets</v>
+        <v>/macropage-connect/help/docs</v>
       </c>
       <c r="D32" t="str">
         <v>JWT required</v>
@@ -1142,21 +1281,33 @@
         <v>Any</v>
       </c>
       <c r="F32" t="str">
-        <v>{ customerId, subject, description?, status?, priority?, assignedTo? }</v>
-      </c>
-      <c r="G32" t="str">
-        <v>Create a ticket</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>{ title, slug, category, order?, tags?: string[], content }</v>
+      </c>
+      <c r="G32" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "title": "How to connect WhatsApp",
+  "slug": "connect-whatsapp",
+  "category": "getting-started",
+  "order": 1,
+  "tags": [
+    "setup"
+  ],
+  "content": "# Steps..."
+}</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Create</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
       <c r="A33" t="str">
-        <v>Support Tickets</v>
+        <v>Help Docs</v>
       </c>
       <c r="B33" t="str">
         <v>PATCH</v>
       </c>
       <c r="C33" t="str">
-        <v>/support/tickets/:id</v>
+        <v>/macropage-connect/help/docs/:id</v>
       </c>
       <c r="D33" t="str">
         <v>JWT required</v>
@@ -1167,19 +1318,24 @@
       <c r="F33" t="str">
         <v>Partial of create body</v>
       </c>
-      <c r="G33" t="str">
-        <v>Update a ticket</v>
+      <c r="G33" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "content": "# Updated steps..."
+}</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Update</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Support Tickets</v>
+        <v>Help Docs</v>
       </c>
       <c r="B34" t="str">
         <v>DELETE</v>
       </c>
       <c r="C34" t="str">
-        <v>/support/tickets/:id</v>
+        <v>/macropage-connect/help/docs/:id</v>
       </c>
       <c r="D34" t="str">
         <v>JWT required</v>
@@ -1191,46 +1347,359 @@
         <v>-</v>
       </c>
       <c r="G34" t="str">
-        <v>Delete a ticket</v>
-      </c>
-    </row>
-    <row r="35" xml:space="preserve">
+        <v>-</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Delete</v>
+      </c>
+    </row>
+    <row r="35">
       <c r="A35" t="str">
-        <v>Support Live Chat</v>
+        <v>Help FAQs</v>
       </c>
       <c r="B35" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C35" t="str">
+        <v>/macropage-connect/help/faqs</v>
+      </c>
+      <c r="D35" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Query: category?</v>
+      </c>
+      <c r="G35" t="str">
+        <v>-</v>
+      </c>
+      <c r="H35" t="str">
+        <v>List FAQs (real, live helpfaqs collection)</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Help FAQs</v>
+      </c>
+      <c r="B36" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C36" t="str">
+        <v>/macropage-connect/help/faqs/:id</v>
+      </c>
+      <c r="D36" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F36" t="str">
+        <v>-</v>
+      </c>
+      <c r="G36" t="str">
+        <v>-</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Get one</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>Help FAQs</v>
+      </c>
+      <c r="B37" t="str">
+        <v>POST</v>
+      </c>
+      <c r="C37" t="str">
+        <v>/macropage-connect/help/faqs</v>
+      </c>
+      <c r="D37" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F37" t="str">
+        <v>{ category, order?, question, answer, tags?: string[] }</v>
+      </c>
+      <c r="G37" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "category": "billing",
+  "question": "How do I cancel my plan?",
+  "answer": "Go to Settings &gt; Billing &gt; Cancel.",
+  "tags": [
+    "billing",
+    "cancel"
+  ]
+}</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Create</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>Help FAQs</v>
+      </c>
+      <c r="B38" t="str">
+        <v>PATCH</v>
+      </c>
+      <c r="C38" t="str">
+        <v>/macropage-connect/help/faqs/:id</v>
+      </c>
+      <c r="D38" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Partial of create body</v>
+      </c>
+      <c r="G38" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "answer": "Updated answer text"
+}</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Update</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Help FAQs</v>
+      </c>
+      <c r="B39" t="str">
+        <v>DELETE</v>
+      </c>
+      <c r="C39" t="str">
+        <v>/macropage-connect/help/faqs/:id</v>
+      </c>
+      <c r="D39" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F39" t="str">
+        <v>-</v>
+      </c>
+      <c r="G39" t="str">
+        <v>-</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Delete</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Upload</v>
+      </c>
+      <c r="B40" t="str">
+        <v>POST</v>
+      </c>
+      <c r="C40" t="str">
+        <v>/macropage-connect/upload/tutorial</v>
+      </c>
+      <c r="D40" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F40" t="str">
+        <v>multipart/form-data, field name "file" (image/jpeg|png|webp|gif, video/mp4|webm, or application/pdf — max 100MB)</v>
+      </c>
+      <c r="G40" t="str">
+        <v>curl -F "file=@tutorial.mp4" .../upload/tutorial</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Uploads to DO Spaces (admin-tutorials/ prefix), returns { url }</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Support Tickets</v>
+      </c>
+      <c r="B41" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C41" t="str">
+        <v>/macropage-connect/support/tickets</v>
+      </c>
+      <c r="D41" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Query: page, limit, status(open|pending|resolved|closed), priority(low|medium|high), customerId, assignedTo</v>
+      </c>
+      <c r="G41" t="str">
+        <v>-</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Paginated list</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Support Tickets</v>
+      </c>
+      <c r="B42" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C42" t="str">
+        <v>/macropage-connect/support/tickets/:id</v>
+      </c>
+      <c r="D42" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F42" t="str">
+        <v>-</v>
+      </c>
+      <c r="G42" t="str">
+        <v>-</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Get one</v>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
+        <v>Support Tickets</v>
+      </c>
+      <c r="B43" t="str">
+        <v>POST</v>
+      </c>
+      <c r="C43" t="str">
+        <v>/macropage-connect/support/tickets</v>
+      </c>
+      <c r="D43" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F43" t="str">
+        <v>{ customerId, subject, description?, status?, priority?, assignedTo? }</v>
+      </c>
+      <c r="G43" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "customerId": "665f1a2b9c1d4e0012345678",
+  "subject": "Cannot connect WhatsApp number",
+  "priority": "high"
+}</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Create</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>Support Tickets</v>
+      </c>
+      <c r="B44" t="str">
+        <v>PATCH</v>
+      </c>
+      <c r="C44" t="str">
+        <v>/macropage-connect/support/tickets/:id</v>
+      </c>
+      <c r="D44" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Partial of create body</v>
+      </c>
+      <c r="G44" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "status": "resolved"
+}</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Update</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Support Tickets</v>
+      </c>
+      <c r="B45" t="str">
+        <v>DELETE</v>
+      </c>
+      <c r="C45" t="str">
+        <v>/macropage-connect/support/tickets/:id</v>
+      </c>
+      <c r="D45" t="str">
+        <v>JWT required</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F45" t="str">
+        <v>-</v>
+      </c>
+      <c r="G45" t="str">
+        <v>-</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Delete</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
+        <v>Live Chat</v>
+      </c>
+      <c r="B46" t="str">
         <v>WS</v>
       </c>
-      <c r="C35" t="str">
-        <v>/support-chat (Socket.io namespace)</v>
-      </c>
-      <c r="D35" t="str">
+      <c r="C46" t="str">
+        <v>/macropage-connect/support-chat</v>
+      </c>
+      <c r="D46" t="str">
         <v>JWT in handshake (auth.token)</v>
       </c>
-      <c r="E35" t="str">
-        <v>Any</v>
-      </c>
-      <c r="F35" t="str" xml:space="preserve">
+      <c r="E46" t="str">
+        <v>Any</v>
+      </c>
+      <c r="F46" t="str" xml:space="preserve">
         <v xml:space="preserve">emit "joinTicket": { ticketId }
-emit "sendMessage": { ticketId, senderType, senderId, message }</v>
-      </c>
-      <c r="G35" t="str">
-        <v>Real-time chat; server emits "history" on join and "newMessage" on send, rooms keyed by ticketId</v>
+emit "sendMessage": { ticketId, senderType(customer|agent), senderId, message }</v>
+      </c>
+      <c r="G46" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "ticketId": "665f...",
+  "senderType": "agent",
+  "senderId": "admin123",
+  "message": "How can I help?"
+}</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Socket.io namespace. Server emits "history" on join, "newMessage" on send.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G35"/>
+  <autoFilter ref="A1:H46"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H46"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <cols>
-    <col min="1" max="1" width="100.83203125" customWidth="1"/>
+    <col min="1" max="1" width="115.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1240,37 +1709,42 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Base URL (local dev): http://localhost:3000/api</v>
+        <v>Base URL (local dev): http://localhost:3000/api — deployed: &lt;your Render URL&gt;/api</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>All routes require "Authorization: Bearer &lt;token&gt;" except POST /auth/login.</v>
+        <v>Every route lives under /api/macropage-connect/* except /api/auth/login, which is SHARED with mr-fuels.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>No route currently restricts by admin role (super-admin vs support-agent) — any logged-in admin can call any endpoint.</v>
+        <v>Successful responses: { success: true, data: ... }. Errors: { success: false, statusCode, path, timestamp, message }.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Successful responses are wrapped as { success: true, data: ... }. Errors: { success: false, statusCode, path, timestamp, message }.</v>
+        <v>Paginated list endpoints return: { items, total, page, limit, totalPages }.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>List endpoints returning "paginated" use shape: { items, total, page, limit, totalPages }.</v>
+        <v>"customerId"/"tenantId" = real "users" collection _id (a WhatsApp SaaS tenant, role OWNER).</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>"customerId" / "tenantId" refer to the real product's user _id (a tenant/customer account with role OWNER).</v>
+        <v>help/docs and help/faqs write into the REAL macropage-connect product's live self-serve help center.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>notifications channel "in_app" writes into the real live "notifications" collection the tenant sees in-app.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>